<commit_message>
Renombrar Dosis I-131 a Dosis Hiper (fuente unica en tipoI131.js), fix 404 de plantilla de turnos, orden correcto de pestanas Libro 1-4 en Actas ARN
</commit_message>
<xml_diff>
--- a/public/plantilla-turnos-i131.xlsx
+++ b/public/plantilla-turnos-i131.xlsx
@@ -503,9 +503,9 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
     <col width="20" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
@@ -521,17 +521,17 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>telefono</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>pacienteNombre</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>pacienteDni</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>telefono</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
@@ -568,22 +568,22 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
+          <t>261-5551234</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
           <t>García Juan</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>28456789</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>261-5551234</t>
-        </is>
-      </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Dosis I-131</t>
+          <t>Dosis Hiper</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -1028,7 +1028,7 @@
   </sheetData>
   <dataValidations count="1">
     <dataValidation sqref="E3:E40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Tipo de dosis inválido" error="Elegí un valor de la lista" type="list">
-      <formula1>"Ablativa I-131,Dosis I-131,Barrido I-131,Captación I-131,Centellograma I-131,Capt.+Centellograma I-131"</formula1>
+      <formula1>"Ablativa I-131,Dosis Hiper,Barrido I-131,Captación I-131,Centellograma I-131,Capt.+Centellograma I-131"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1129,21 +1129,21 @@
     <row r="14" ht="20" customHeight="1">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>pacienteNombre — Nombre y apellido del paciente. Obligatorio.</t>
+          <t>telefono — Teléfono de contacto. Opcional.</t>
         </is>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>pacienteDni — Solo números, sin puntos ni espacios. Obligatorio.</t>
+          <t>pacienteNombre — Nombre y apellido del paciente. Obligatorio.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="20" customHeight="1">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>telefono — Teléfono de contacto. Opcional.</t>
+          <t>pacienteDni — Solo números, sin puntos ni espacios. Obligatorio.</t>
         </is>
       </c>
     </row>

</xml_diff>